<commit_message>
Comprobacion en agregar pedido
</commit_message>
<xml_diff>
--- a/019-085-WENDLANDT-VENTAS/src/WendlandtVentas.Web/wwwroot/resources/Cotizacion - Factura.xlsx
+++ b/019-085-WENDLANDT-VENTAS/src/WendlandtVentas.Web/wwwroot/resources/Cotizacion - Factura.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WENDLANDT SYS\Wend-Sys\019-085-WENDLANDT-VENTAS\src\WendlandtVentas.Web\wwwroot\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01E9F78E-6726-4F40-96CF-DA8CFBF158C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21EA1884-CF50-4A95-9B66-AE1B8C9DD209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1F49A7E6-679B-4399-A417-11073B80C7DF}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1F49A7E6-679B-4399-A417-11073B80C7DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>CANT</t>
   </si>
@@ -110,6 +110,12 @@
   </si>
   <si>
     <t>Cotizacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>*Pedido sujeto a disponibilidad de inventario al momento de su preparación.</t>
   </si>
 </sst>
 </file>
@@ -218,7 +224,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -340,25 +346,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -374,6 +367,12 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -434,9 +433,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -518,14 +514,62 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -587,55 +631,6 @@
         <a:xfrm>
           <a:off x="7620" y="114301"/>
           <a:ext cx="1371600" cy="622934"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>411481</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>22861</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>388621</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>118873</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D71E4F9E-855B-4CE7-8FA0-091C0613EABF}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="22031" r="21250"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4480561" y="137161"/>
-          <a:ext cx="1371600" cy="621792"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -983,156 +978,136 @@
       <c r="A2" s="4"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
-      <c r="D2" s="42" t="s">
+      <c r="D2" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
       <c r="G2" s="4"/>
-      <c r="H2" s="47" t="s">
+      <c r="H2" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="48"/>
-      <c r="J2" s="49"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="42" t="s">
-        <v>7</v>
-      </c>
-      <c r="O2" s="42"/>
-      <c r="P2" s="42"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="47" t="s">
-        <v>27</v>
-      </c>
-      <c r="S2" s="48"/>
-      <c r="T2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="50"/>
+      <c r="L2" s="59"/>
+      <c r="M2" s="59"/>
+      <c r="N2" s="60"/>
+      <c r="O2" s="60"/>
+      <c r="P2" s="60"/>
+      <c r="Q2" s="59"/>
+      <c r="R2" s="61"/>
+      <c r="S2" s="61"/>
+      <c r="T2" s="61"/>
     </row>
     <row r="3" spans="1:20" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
-      <c r="D3" s="42" t="s">
+      <c r="D3" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
       <c r="G3" s="4"/>
-      <c r="H3" s="50">
+      <c r="H3" s="51">
         <v>5932</v>
       </c>
-      <c r="I3" s="51"/>
-      <c r="J3" s="52"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="42" t="s">
-        <v>8</v>
-      </c>
-      <c r="O3" s="42"/>
-      <c r="P3" s="42"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="50">
-        <v>5932</v>
-      </c>
-      <c r="S3" s="51"/>
-      <c r="T3" s="52"/>
+      <c r="I3" s="52"/>
+      <c r="J3" s="53"/>
+      <c r="L3" s="59"/>
+      <c r="M3" s="59"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="62"/>
+      <c r="S3" s="62"/>
+      <c r="T3" s="62"/>
     </row>
     <row r="4" spans="1:20" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
-      <c r="D4" s="42" t="s">
+      <c r="D4" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
       <c r="G4" s="4"/>
-      <c r="H4" s="53" t="s">
+      <c r="H4" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="54"/>
-      <c r="J4" s="55"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="42" t="s">
-        <v>9</v>
-      </c>
-      <c r="O4" s="42"/>
-      <c r="P4" s="42"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="53" t="s">
-        <v>22</v>
-      </c>
-      <c r="S4" s="54"/>
-      <c r="T4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="56"/>
+      <c r="L4" s="59"/>
+      <c r="M4" s="59"/>
+      <c r="N4" s="60"/>
+      <c r="O4" s="60"/>
+      <c r="P4" s="60"/>
+      <c r="Q4" s="59"/>
+      <c r="R4" s="61"/>
+      <c r="S4" s="61"/>
+      <c r="T4" s="61"/>
     </row>
     <row r="5" spans="1:20" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
-      <c r="D5" s="42" t="s">
+      <c r="D5" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="50">
+      <c r="H5" s="51">
         <v>2020000033</v>
       </c>
-      <c r="I5" s="51"/>
-      <c r="J5" s="52"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="42" t="s">
-        <v>10</v>
-      </c>
-      <c r="O5" s="42"/>
-      <c r="P5" s="42"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="50">
-        <v>2020000033</v>
-      </c>
-      <c r="S5" s="51"/>
-      <c r="T5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="53"/>
+      <c r="L5" s="59"/>
+      <c r="M5" s="59"/>
+      <c r="N5" s="60"/>
+      <c r="O5" s="60"/>
+      <c r="P5" s="60"/>
+      <c r="Q5" s="59"/>
+      <c r="R5" s="62"/>
+      <c r="S5" s="62"/>
+      <c r="T5" s="62"/>
     </row>
     <row r="6" spans="1:20" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
-      <c r="D6" s="42" t="s">
+      <c r="D6" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="56" t="s">
+      <c r="H6" s="57" t="s">
         <v>4</v>
       </c>
-      <c r="I6" s="56"/>
-      <c r="J6" s="56"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="42" t="s">
-        <v>11</v>
-      </c>
-      <c r="O6" s="42"/>
-      <c r="P6" s="42"/>
-      <c r="Q6" s="4"/>
-      <c r="R6" s="56" t="s">
-        <v>4</v>
-      </c>
-      <c r="S6" s="56"/>
-      <c r="T6" s="56"/>
+      <c r="I6" s="57"/>
+      <c r="J6" s="57"/>
+      <c r="L6" s="59"/>
+      <c r="M6" s="59"/>
+      <c r="N6" s="60"/>
+      <c r="O6" s="60"/>
+      <c r="P6" s="60"/>
+      <c r="Q6" s="59"/>
+      <c r="R6" s="63"/>
+      <c r="S6" s="63"/>
+      <c r="T6" s="63"/>
     </row>
     <row r="7" spans="1:20" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="44"/>
       <c r="G7" s="4"/>
       <c r="H7" s="6" t="s">
         <v>21</v>
@@ -1143,23 +1118,15 @@
       <c r="J7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="43" t="s">
-        <v>12</v>
-      </c>
-      <c r="O7" s="43"/>
-      <c r="P7" s="43"/>
-      <c r="Q7" s="4"/>
-      <c r="R7" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="S7" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="T7" s="6" t="s">
-        <v>6</v>
-      </c>
+      <c r="L7" s="59"/>
+      <c r="M7" s="59"/>
+      <c r="N7" s="61"/>
+      <c r="O7" s="61"/>
+      <c r="P7" s="61"/>
+      <c r="Q7" s="59"/>
+      <c r="R7" s="64"/>
+      <c r="S7" s="64"/>
+      <c r="T7" s="64"/>
     </row>
     <row r="8" spans="1:20" ht="9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
@@ -1172,618 +1139,556 @@
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
-      <c r="P8" s="4"/>
-      <c r="Q8" s="4"/>
-      <c r="R8" s="4"/>
-      <c r="S8" s="4"/>
-      <c r="T8" s="4"/>
+      <c r="L8" s="59"/>
+      <c r="M8" s="59"/>
+      <c r="N8" s="59"/>
+      <c r="O8" s="59"/>
+      <c r="P8" s="59"/>
+      <c r="Q8" s="59"/>
+      <c r="R8" s="59"/>
+      <c r="S8" s="59"/>
+      <c r="T8" s="59"/>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="B9" s="44" t="s">
+      <c r="B9" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="45"/>
-      <c r="D9" s="45"/>
-      <c r="E9" s="45"/>
-      <c r="F9" s="45"/>
-      <c r="G9" s="45"/>
-      <c r="H9" s="45"/>
-      <c r="I9" s="45"/>
-      <c r="J9" s="46"/>
-      <c r="L9" s="44" t="s">
-        <v>20</v>
-      </c>
-      <c r="M9" s="45"/>
-      <c r="N9" s="45"/>
-      <c r="O9" s="45"/>
-      <c r="P9" s="45"/>
-      <c r="Q9" s="45"/>
-      <c r="R9" s="45"/>
-      <c r="S9" s="45"/>
-      <c r="T9" s="46"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="46"/>
+      <c r="J9" s="47"/>
+      <c r="L9" s="65"/>
+      <c r="M9" s="65"/>
+      <c r="N9" s="65"/>
+      <c r="O9" s="65"/>
+      <c r="P9" s="65"/>
+      <c r="Q9" s="65"/>
+      <c r="R9" s="65"/>
+      <c r="S9" s="65"/>
+      <c r="T9" s="65"/>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="45" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="45"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="45"/>
-      <c r="F10" s="45"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="45"/>
-      <c r="I10" s="45"/>
-      <c r="J10" s="46"/>
-      <c r="L10" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="M10" s="45"/>
-      <c r="N10" s="45"/>
-      <c r="O10" s="45"/>
-      <c r="P10" s="45"/>
-      <c r="Q10" s="45"/>
-      <c r="R10" s="45"/>
-      <c r="S10" s="45"/>
-      <c r="T10" s="46"/>
+      <c r="C10" s="46"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="46"/>
+      <c r="J10" s="47"/>
+      <c r="L10" s="65"/>
+      <c r="M10" s="65"/>
+      <c r="N10" s="65"/>
+      <c r="O10" s="65"/>
+      <c r="P10" s="65"/>
+      <c r="Q10" s="65"/>
+      <c r="R10" s="65"/>
+      <c r="S10" s="65"/>
+      <c r="T10" s="65"/>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
-      <c r="B11" s="44" t="s">
+      <c r="B11" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="45"/>
-      <c r="F11" s="45"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="45" t="s">
+      <c r="C11" s="46"/>
+      <c r="D11" s="46"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="45"/>
-      <c r="J11" s="46"/>
-      <c r="L11" s="44" t="s">
-        <v>18</v>
-      </c>
-      <c r="M11" s="45"/>
-      <c r="N11" s="45"/>
-      <c r="O11" s="45"/>
-      <c r="P11" s="45"/>
-      <c r="Q11" s="45"/>
-      <c r="R11" s="45" t="s">
-        <v>17</v>
-      </c>
-      <c r="S11" s="45"/>
-      <c r="T11" s="46"/>
+      <c r="I11" s="46"/>
+      <c r="J11" s="47"/>
+      <c r="L11" s="65"/>
+      <c r="M11" s="65"/>
+      <c r="N11" s="65"/>
+      <c r="O11" s="65"/>
+      <c r="P11" s="65"/>
+      <c r="Q11" s="65"/>
+      <c r="R11" s="65"/>
+      <c r="S11" s="65"/>
+      <c r="T11" s="65"/>
     </row>
     <row r="12" spans="1:20" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
-      <c r="P12" s="4"/>
-      <c r="Q12" s="4"/>
-      <c r="R12" s="4"/>
-      <c r="S12" s="4"/>
-      <c r="T12" s="4"/>
+      <c r="L12" s="59"/>
+      <c r="M12" s="59"/>
+      <c r="N12" s="59"/>
+      <c r="O12" s="59"/>
+      <c r="P12" s="59"/>
+      <c r="Q12" s="59"/>
+      <c r="R12" s="59"/>
+      <c r="S12" s="59"/>
+      <c r="T12" s="59"/>
     </row>
     <row r="13" spans="1:20" ht="26.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C13" s="37" t="s">
+      <c r="C13" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="38"/>
-      <c r="G13" s="40" t="s">
+      <c r="D13" s="40"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="H13" s="41"/>
-      <c r="I13" s="37" t="s">
+      <c r="H13" s="42"/>
+      <c r="I13" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="J13" s="38"/>
-      <c r="L13" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="M13" s="37" t="s">
-        <v>1</v>
-      </c>
-      <c r="N13" s="39"/>
-      <c r="O13" s="39"/>
-      <c r="P13" s="38"/>
-      <c r="Q13" s="40" t="s">
-        <v>2</v>
-      </c>
-      <c r="R13" s="41"/>
-      <c r="S13" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="T13" s="38"/>
+      <c r="J13" s="39"/>
+      <c r="L13" s="64"/>
+      <c r="M13" s="66"/>
+      <c r="N13" s="66"/>
+      <c r="O13" s="66"/>
+      <c r="P13" s="66"/>
+      <c r="Q13" s="67"/>
+      <c r="R13" s="67"/>
+      <c r="S13" s="66"/>
+      <c r="T13" s="66"/>
     </row>
     <row r="14" spans="1:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B14" s="3"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="18"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="12"/>
-      <c r="N14" s="13"/>
-      <c r="O14" s="13"/>
-      <c r="P14" s="14"/>
-      <c r="Q14" s="15"/>
-      <c r="R14" s="16"/>
-      <c r="S14" s="17"/>
-      <c r="T14" s="18"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="20"/>
+      <c r="L14" s="68"/>
+      <c r="M14" s="69"/>
+      <c r="N14" s="69"/>
+      <c r="O14" s="69"/>
+      <c r="P14" s="69"/>
+      <c r="Q14" s="70"/>
+      <c r="R14" s="70"/>
+      <c r="S14" s="71"/>
+      <c r="T14" s="71"/>
     </row>
     <row r="15" spans="1:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B15" s="3"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="18"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="12"/>
-      <c r="N15" s="13"/>
-      <c r="O15" s="13"/>
-      <c r="P15" s="14"/>
-      <c r="Q15" s="15"/>
-      <c r="R15" s="16"/>
-      <c r="S15" s="17"/>
-      <c r="T15" s="18"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="19"/>
+      <c r="J15" s="20"/>
+      <c r="L15" s="68"/>
+      <c r="M15" s="69"/>
+      <c r="N15" s="69"/>
+      <c r="O15" s="69"/>
+      <c r="P15" s="69"/>
+      <c r="Q15" s="70"/>
+      <c r="R15" s="70"/>
+      <c r="S15" s="71"/>
+      <c r="T15" s="71"/>
     </row>
     <row r="16" spans="1:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B16" s="3"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="16"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="18"/>
-      <c r="L16" s="3"/>
-      <c r="M16" s="12"/>
-      <c r="N16" s="13"/>
-      <c r="O16" s="13"/>
-      <c r="P16" s="14"/>
-      <c r="Q16" s="15"/>
-      <c r="R16" s="16"/>
-      <c r="S16" s="17"/>
-      <c r="T16" s="18"/>
-    </row>
-    <row r="17" spans="2:21" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="C16" s="14"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="20"/>
+      <c r="L16" s="68"/>
+      <c r="M16" s="69"/>
+      <c r="N16" s="69"/>
+      <c r="O16" s="69"/>
+      <c r="P16" s="69"/>
+      <c r="Q16" s="70"/>
+      <c r="R16" s="70"/>
+      <c r="S16" s="71"/>
+      <c r="T16" s="71"/>
+    </row>
+    <row r="17" spans="2:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B17" s="3"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="18"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="12"/>
-      <c r="N17" s="13"/>
-      <c r="O17" s="13"/>
-      <c r="P17" s="14"/>
-      <c r="Q17" s="15"/>
-      <c r="R17" s="16"/>
-      <c r="S17" s="17"/>
-      <c r="T17" s="18"/>
-    </row>
-    <row r="18" spans="2:21" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="C17" s="14"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="20"/>
+      <c r="L17" s="68"/>
+      <c r="M17" s="69"/>
+      <c r="N17" s="69"/>
+      <c r="O17" s="69"/>
+      <c r="P17" s="69"/>
+      <c r="Q17" s="70"/>
+      <c r="R17" s="70"/>
+      <c r="S17" s="71"/>
+      <c r="T17" s="71"/>
+    </row>
+    <row r="18" spans="2:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B18" s="3"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="18"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="12"/>
-      <c r="N18" s="13"/>
-      <c r="O18" s="13"/>
-      <c r="P18" s="14"/>
-      <c r="Q18" s="15"/>
-      <c r="R18" s="16"/>
-      <c r="S18" s="17"/>
-      <c r="T18" s="18"/>
-    </row>
-    <row r="19" spans="2:21" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="C18" s="14"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="20"/>
+      <c r="L18" s="68"/>
+      <c r="M18" s="69"/>
+      <c r="N18" s="69"/>
+      <c r="O18" s="69"/>
+      <c r="P18" s="69"/>
+      <c r="Q18" s="70"/>
+      <c r="R18" s="70"/>
+      <c r="S18" s="71"/>
+      <c r="T18" s="71"/>
+    </row>
+    <row r="19" spans="2:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B19" s="3"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="18"/>
-      <c r="L19" s="3"/>
-      <c r="M19" s="12"/>
-      <c r="N19" s="13"/>
-      <c r="O19" s="13"/>
-      <c r="P19" s="14"/>
-      <c r="Q19" s="15"/>
-      <c r="R19" s="16"/>
-      <c r="S19" s="17"/>
-      <c r="T19" s="18"/>
-    </row>
-    <row r="20" spans="2:21" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="C19" s="14"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="20"/>
+      <c r="L19" s="68"/>
+      <c r="M19" s="69"/>
+      <c r="N19" s="69"/>
+      <c r="O19" s="69"/>
+      <c r="P19" s="69"/>
+      <c r="Q19" s="70"/>
+      <c r="R19" s="70"/>
+      <c r="S19" s="71"/>
+      <c r="T19" s="71"/>
+    </row>
+    <row r="20" spans="2:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B20" s="3"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="18"/>
-      <c r="L20" s="3"/>
-      <c r="M20" s="12"/>
-      <c r="N20" s="13"/>
-      <c r="O20" s="13"/>
-      <c r="P20" s="14"/>
-      <c r="Q20" s="15"/>
-      <c r="R20" s="16"/>
-      <c r="S20" s="17"/>
-      <c r="T20" s="18"/>
-    </row>
-    <row r="21" spans="2:21" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="C20" s="14"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="20"/>
+      <c r="L20" s="68"/>
+      <c r="M20" s="69"/>
+      <c r="N20" s="69"/>
+      <c r="O20" s="69"/>
+      <c r="P20" s="69"/>
+      <c r="Q20" s="70"/>
+      <c r="R20" s="70"/>
+      <c r="S20" s="71"/>
+      <c r="T20" s="71"/>
+    </row>
+    <row r="21" spans="2:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B21" s="3"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="16"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="18"/>
-      <c r="L21" s="3"/>
-      <c r="M21" s="12"/>
-      <c r="N21" s="13"/>
-      <c r="O21" s="13"/>
-      <c r="P21" s="14"/>
-      <c r="Q21" s="15"/>
-      <c r="R21" s="16"/>
-      <c r="S21" s="17"/>
-      <c r="T21" s="18"/>
-    </row>
-    <row r="22" spans="2:21" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="C21" s="14"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="19"/>
+      <c r="J21" s="20"/>
+      <c r="L21" s="68"/>
+      <c r="M21" s="69"/>
+      <c r="N21" s="69"/>
+      <c r="O21" s="69"/>
+      <c r="P21" s="69"/>
+      <c r="Q21" s="70"/>
+      <c r="R21" s="70"/>
+      <c r="S21" s="71"/>
+      <c r="T21" s="71"/>
+    </row>
+    <row r="22" spans="2:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B22" s="3"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="18"/>
-      <c r="L22" s="3"/>
-      <c r="M22" s="12"/>
-      <c r="N22" s="13"/>
-      <c r="O22" s="13"/>
-      <c r="P22" s="14"/>
-      <c r="Q22" s="15"/>
-      <c r="R22" s="16"/>
-      <c r="S22" s="17"/>
-      <c r="T22" s="18"/>
-    </row>
-    <row r="23" spans="2:21" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="C22" s="14"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="20"/>
+      <c r="L22" s="68"/>
+      <c r="M22" s="69"/>
+      <c r="N22" s="69"/>
+      <c r="O22" s="69"/>
+      <c r="P22" s="69"/>
+      <c r="Q22" s="70"/>
+      <c r="R22" s="70"/>
+      <c r="S22" s="71"/>
+      <c r="T22" s="71"/>
+    </row>
+    <row r="23" spans="2:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B23" s="3"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="16"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="18"/>
-      <c r="L23" s="3"/>
-      <c r="M23" s="12"/>
-      <c r="N23" s="13"/>
-      <c r="O23" s="13"/>
-      <c r="P23" s="14"/>
-      <c r="Q23" s="15"/>
-      <c r="R23" s="16"/>
-      <c r="S23" s="17"/>
-      <c r="T23" s="18"/>
-    </row>
-    <row r="24" spans="2:21" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="C23" s="14"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="20"/>
+      <c r="L23" s="68"/>
+      <c r="M23" s="69"/>
+      <c r="N23" s="69"/>
+      <c r="O23" s="69"/>
+      <c r="P23" s="69"/>
+      <c r="Q23" s="70"/>
+      <c r="R23" s="70"/>
+      <c r="S23" s="71"/>
+      <c r="T23" s="71"/>
+    </row>
+    <row r="24" spans="2:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B24" s="3"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="16"/>
-      <c r="I24" s="17"/>
-      <c r="J24" s="18"/>
-      <c r="L24" s="3"/>
-      <c r="M24" s="12"/>
-      <c r="N24" s="13"/>
-      <c r="O24" s="13"/>
-      <c r="P24" s="14"/>
-      <c r="Q24" s="15"/>
-      <c r="R24" s="16"/>
-      <c r="S24" s="17"/>
-      <c r="T24" s="18"/>
-    </row>
-    <row r="25" spans="2:21" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="B25" s="19" t="s">
+      <c r="C24" s="14"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="19"/>
+      <c r="J24" s="20"/>
+      <c r="L24" s="68"/>
+      <c r="M24" s="69"/>
+      <c r="N24" s="69"/>
+      <c r="O24" s="69"/>
+      <c r="P24" s="69"/>
+      <c r="Q24" s="70"/>
+      <c r="R24" s="70"/>
+      <c r="S24" s="71"/>
+      <c r="T24" s="71"/>
+    </row>
+    <row r="25" spans="2:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="B25" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="C25" s="20"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="18"/>
-      <c r="L25" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="M25" s="20"/>
-      <c r="N25" s="23"/>
-      <c r="O25" s="24"/>
-      <c r="P25" s="25"/>
-      <c r="Q25" s="15"/>
-      <c r="R25" s="16"/>
-      <c r="S25" s="17"/>
-      <c r="T25" s="18"/>
-    </row>
-    <row r="26" spans="2:21" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="B26" s="21"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="27"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="18"/>
-      <c r="L26" s="21"/>
-      <c r="M26" s="22"/>
-      <c r="N26" s="26"/>
-      <c r="O26" s="27"/>
-      <c r="P26" s="28"/>
-      <c r="Q26" s="15"/>
-      <c r="R26" s="16"/>
-      <c r="S26" s="17"/>
-      <c r="T26" s="18"/>
-    </row>
-    <row r="27" spans="2:21" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="B27" s="31" t="s">
+      <c r="C25" s="22"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="19"/>
+      <c r="J25" s="20"/>
+      <c r="L25" s="72"/>
+      <c r="M25" s="72"/>
+      <c r="N25" s="73"/>
+      <c r="O25" s="73"/>
+      <c r="P25" s="73"/>
+      <c r="Q25" s="70"/>
+      <c r="R25" s="70"/>
+      <c r="S25" s="71"/>
+      <c r="T25" s="71"/>
+    </row>
+    <row r="26" spans="2:20" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="B26" s="23"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="30"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="19"/>
+      <c r="J26" s="20"/>
+      <c r="L26" s="72"/>
+      <c r="M26" s="72"/>
+      <c r="N26" s="73"/>
+      <c r="O26" s="73"/>
+      <c r="P26" s="73"/>
+      <c r="Q26" s="70"/>
+      <c r="R26" s="70"/>
+      <c r="S26" s="71"/>
+      <c r="T26" s="71"/>
+    </row>
+    <row r="27" spans="2:20" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="B27" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="C27" s="31"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="11" t="s">
+      <c r="C27" s="32"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="H27" s="11"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-      <c r="L27" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="M27" s="31"/>
-      <c r="N27" s="32"/>
-      <c r="O27" s="32"/>
-      <c r="P27" s="32"/>
-      <c r="Q27" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="R27" s="11"/>
-      <c r="S27" s="9"/>
-      <c r="T27" s="9"/>
-    </row>
-    <row r="28" spans="2:21" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="B28" s="31"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="35" t="s">
+      <c r="H27" s="13"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="11"/>
+      <c r="L27" s="74"/>
+      <c r="M27" s="74"/>
+      <c r="N27" s="72"/>
+      <c r="O27" s="72"/>
+      <c r="P27" s="72"/>
+      <c r="Q27" s="66"/>
+      <c r="R27" s="66"/>
+      <c r="S27" s="75"/>
+      <c r="T27" s="75"/>
+    </row>
+    <row r="28" spans="2:20" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="B28" s="32"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="H28" s="10"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="34"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="32"/>
-      <c r="O28" s="32"/>
-      <c r="P28" s="32"/>
-      <c r="Q28" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="R28" s="11"/>
-      <c r="S28" s="9"/>
-      <c r="T28" s="9"/>
-    </row>
-    <row r="29" spans="2:21" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="B29" s="31" t="s">
+      <c r="H28" s="12"/>
+      <c r="I28" s="34"/>
+      <c r="J28" s="35"/>
+      <c r="L28" s="74"/>
+      <c r="M28" s="74"/>
+      <c r="N28" s="72"/>
+      <c r="O28" s="72"/>
+      <c r="P28" s="72"/>
+      <c r="Q28" s="66"/>
+      <c r="R28" s="66"/>
+      <c r="S28" s="75"/>
+      <c r="T28" s="75"/>
+    </row>
+    <row r="29" spans="2:20" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="B29" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="C29" s="31"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="32"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="35" t="s">
+      <c r="C29" s="32"/>
+      <c r="D29" s="33"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="33"/>
+      <c r="G29" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="H29" s="10"/>
-      <c r="I29" s="9"/>
-      <c r="J29" s="9"/>
-      <c r="L29" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="M29" s="31"/>
-      <c r="N29" s="32"/>
-      <c r="O29" s="32"/>
-      <c r="P29" s="32"/>
-      <c r="Q29" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="R29" s="11"/>
-      <c r="S29" s="9"/>
-      <c r="T29" s="9"/>
-    </row>
-    <row r="30" spans="2:21" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="B30" s="31"/>
-      <c r="C30" s="31"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="30" t="s">
+      <c r="H29" s="12"/>
+      <c r="I29" s="11"/>
+      <c r="J29" s="11"/>
+      <c r="L29" s="74"/>
+      <c r="M29" s="74"/>
+      <c r="N29" s="72"/>
+      <c r="O29" s="72"/>
+      <c r="P29" s="72"/>
+      <c r="Q29" s="66"/>
+      <c r="R29" s="66"/>
+      <c r="S29" s="75"/>
+      <c r="T29" s="75"/>
+    </row>
+    <row r="30" spans="2:20" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="B30" s="32"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="33"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="H30" s="30"/>
-      <c r="I30" s="33"/>
-      <c r="J30" s="34"/>
-      <c r="L30" s="31"/>
-      <c r="M30" s="31"/>
-      <c r="N30" s="32"/>
-      <c r="O30" s="32"/>
-      <c r="P30" s="32"/>
-      <c r="Q30" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="R30" s="30"/>
-      <c r="S30" s="9"/>
-      <c r="T30" s="9"/>
-    </row>
-    <row r="31" spans="2:21" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="B31" s="31" t="s">
+      <c r="H30" s="31"/>
+      <c r="I30" s="34"/>
+      <c r="J30" s="35"/>
+      <c r="L30" s="74"/>
+      <c r="M30" s="74"/>
+      <c r="N30" s="72"/>
+      <c r="O30" s="72"/>
+      <c r="P30" s="72"/>
+      <c r="Q30" s="61"/>
+      <c r="R30" s="61"/>
+      <c r="S30" s="75"/>
+      <c r="T30" s="75"/>
+    </row>
+    <row r="31" spans="2:20" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="B31" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="C31" s="57"/>
-      <c r="D31" s="58"/>
-      <c r="E31" s="36"/>
-      <c r="F31" s="58"/>
-      <c r="L31" s="57" t="s">
-        <v>25</v>
-      </c>
-      <c r="M31" s="57"/>
-      <c r="N31" s="58"/>
-      <c r="O31" s="58"/>
-      <c r="P31" s="58"/>
-    </row>
-    <row r="32" spans="2:21" ht="29.45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="7"/>
-      <c r="C32" s="59"/>
-      <c r="D32" s="59"/>
-      <c r="F32" s="60"/>
-      <c r="G32" s="59"/>
-      <c r="H32" s="59"/>
-      <c r="I32" s="59"/>
-      <c r="J32" s="59"/>
-      <c r="K32" s="59"/>
-      <c r="L32" s="60"/>
-      <c r="M32" s="59"/>
-      <c r="N32" s="59"/>
-      <c r="O32" s="59"/>
-      <c r="P32" s="60"/>
-      <c r="Q32" s="59"/>
-      <c r="R32" s="59"/>
-      <c r="S32" s="59"/>
-      <c r="T32" s="59"/>
-      <c r="U32" s="59"/>
-    </row>
-    <row r="33" spans="2:25" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="7"/>
-      <c r="C33" s="60"/>
-      <c r="D33" s="59"/>
-      <c r="F33" s="60"/>
-      <c r="G33" s="60"/>
-      <c r="H33" s="59"/>
-      <c r="I33" s="59"/>
-      <c r="J33" s="59"/>
-      <c r="K33" s="59"/>
-      <c r="L33" s="60"/>
-      <c r="M33" s="60"/>
-      <c r="N33" s="59"/>
-      <c r="O33" s="59"/>
-      <c r="P33" s="60"/>
-      <c r="Q33" s="60"/>
-      <c r="R33" s="59"/>
-      <c r="S33" s="59"/>
-      <c r="T33" s="59"/>
-      <c r="U33" s="59"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="37"/>
+      <c r="F31" s="37"/>
+      <c r="L31" s="74"/>
+      <c r="M31" s="74"/>
+      <c r="N31" s="60"/>
+      <c r="O31" s="60"/>
+      <c r="P31" s="60"/>
+      <c r="Q31" s="59"/>
+      <c r="R31" s="59"/>
+      <c r="S31" s="59"/>
+      <c r="T31" s="59"/>
+    </row>
+    <row r="32" spans="2:20" ht="9.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="58" t="s">
+        <v>29</v>
+      </c>
+      <c r="C32" s="58"/>
+      <c r="D32" s="58"/>
+      <c r="E32" s="58"/>
+      <c r="F32" s="58"/>
+      <c r="G32" s="58"/>
+      <c r="H32" s="58"/>
+      <c r="L32" s="76"/>
+      <c r="M32" s="76"/>
+      <c r="N32" s="76"/>
+      <c r="O32" s="76"/>
+      <c r="P32" s="76"/>
+      <c r="Q32" s="76"/>
+      <c r="R32" s="76"/>
+      <c r="S32" s="77"/>
+      <c r="T32" s="77"/>
+    </row>
+    <row r="33" spans="2:25" ht="10.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="7"/>
+      <c r="L33" s="7"/>
+      <c r="M33" s="10"/>
+      <c r="N33" s="10"/>
+      <c r="O33" s="10"/>
+      <c r="P33" s="10"/>
+      <c r="Q33" s="7"/>
     </row>
     <row r="34" spans="2:25" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="7"/>
-      <c r="C34" s="60"/>
-      <c r="D34" s="59"/>
-      <c r="F34" s="60"/>
-      <c r="G34" s="60"/>
-      <c r="H34" s="59"/>
-      <c r="I34" s="59"/>
-      <c r="J34" s="59"/>
-      <c r="K34" s="59"/>
-      <c r="L34" s="60"/>
-      <c r="M34" s="60"/>
-      <c r="N34" s="59"/>
-      <c r="O34" s="59"/>
-      <c r="P34" s="60"/>
-      <c r="Q34" s="60"/>
-      <c r="R34" s="59"/>
-      <c r="S34" s="59"/>
-      <c r="T34" s="59"/>
-      <c r="U34" s="59"/>
-    </row>
-    <row r="35" spans="2:25" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F35" s="59"/>
-      <c r="G35" s="59"/>
-      <c r="H35" s="59"/>
-      <c r="I35" s="59"/>
-      <c r="J35" s="59"/>
-      <c r="K35" s="59"/>
-      <c r="L35" s="59"/>
-      <c r="M35" s="59"/>
-      <c r="N35" s="59"/>
-      <c r="O35" s="59"/>
-      <c r="P35" s="59"/>
-      <c r="Q35" s="59"/>
-      <c r="R35" s="59"/>
-      <c r="S35" s="59"/>
-      <c r="T35" s="59"/>
-      <c r="U35" s="59"/>
-    </row>
+      <c r="C34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
+      <c r="L34" s="7"/>
+      <c r="M34" s="7"/>
+      <c r="P34" s="7"/>
+      <c r="Q34" s="7"/>
+    </row>
+    <row r="35" spans="2:25" ht="13.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="36" spans="2:25" ht="13.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="Y36" s="8"/>
     </row>
@@ -1809,22 +1714,9 @@
     <row r="63" ht="8.4499999999999993" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="64" ht="8.4499999999999993" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="142">
-    <mergeCell ref="B27:C28"/>
-    <mergeCell ref="D27:F28"/>
-    <mergeCell ref="B29:C30"/>
-    <mergeCell ref="D29:F30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="B25:C26"/>
-    <mergeCell ref="D25:F26"/>
+  <mergeCells count="147">
+    <mergeCell ref="B32:H32"/>
+    <mergeCell ref="L32:R32"/>
     <mergeCell ref="H4:J4"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="H3:J3"/>
@@ -1894,7 +1786,7 @@
     <mergeCell ref="Q18:R18"/>
     <mergeCell ref="S18:T18"/>
     <mergeCell ref="I18:J18"/>
-    <mergeCell ref="Q22:R22"/>
+    <mergeCell ref="G18:H18"/>
     <mergeCell ref="S22:T22"/>
     <mergeCell ref="M23:P23"/>
     <mergeCell ref="Q23:R23"/>
@@ -1914,7 +1806,6 @@
     <mergeCell ref="Q21:R21"/>
     <mergeCell ref="S21:T21"/>
     <mergeCell ref="M22:P22"/>
-    <mergeCell ref="Q30:R30"/>
     <mergeCell ref="S30:T30"/>
     <mergeCell ref="L27:M28"/>
     <mergeCell ref="L29:M30"/>
@@ -1938,10 +1829,7 @@
     <mergeCell ref="N31:P31"/>
     <mergeCell ref="Q26:R26"/>
     <mergeCell ref="S26:T26"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="Q27:R27"/>
-    <mergeCell ref="M24:P24"/>
-    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="B27:C28"/>
     <mergeCell ref="S27:T27"/>
     <mergeCell ref="Q28:R28"/>
     <mergeCell ref="S28:T28"/>
@@ -1952,6 +1840,28 @@
     <mergeCell ref="S25:T25"/>
     <mergeCell ref="L25:M26"/>
     <mergeCell ref="N25:P26"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="M33:P33"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="M24:P24"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="Q30:R30"/>
+    <mergeCell ref="Q22:R22"/>
+    <mergeCell ref="D27:F28"/>
+    <mergeCell ref="B29:C30"/>
+    <mergeCell ref="D29:F30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="B25:C26"/>
+    <mergeCell ref="D25:F26"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>